<commit_message>
Office export from plain photos: flatten, high-res reading, line rereads
- Photos of a page on a desk are flattened like a scan (page detection,
  perspective, paper cleanup) and snapped to Letter/A4 before rebuilding
- Text is recognized from a higher-resolution copy; every line and table
  cell is reread on its own and accepted only for plausible corrections
- Page-relative bold threshold, stricter bullet dots, list items no longer
  swallow the next item, "81" → "B1" in code columns, consistent ranges
- Raw photo fixture and test with rendered outputs

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2KPqXq9Whv7eR2vrvkBWC
</commit_message>
<xml_diff>
--- a/ios/Verification/office-layout/OfficeSamplePriceList.xlsx
+++ b/ios/Verification/office-layout/OfficeSamplePriceList.xlsx
@@ -608,7 +608,7 @@
               <rFont val="Arial"/>
               <family val="2"/>
             </rPr>
-            <t xml:space="preserve"> trust'.</t>
+            <t xml:space="preserve"> trust.</t>
           </r>
         </is>
       </c>
@@ -652,7 +652,7 @@
       </c>
       <c r="I35" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONCERT</t>
+          <t xml:space="preserve">CONCERT®</t>
         </is>
       </c>
     </row>

</xml_diff>